<commit_message>
Weekly update for August 31, 2026
</commit_message>
<xml_diff>
--- a/jdca_weekly_metrics_asof_2026-08-31.xlsx
+++ b/jdca_weekly_metrics_asof_2026-08-31.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Job Hunt\Juvenile Diabetes Cure Alliance\Weekly Tracker\Git\jdca-portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CBB865-C057-47CB-92A7-E8C8CA51DF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681F5762-8002-43B4-90E9-918F0861D333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31530" yWindow="840" windowWidth="24750" windowHeight="15405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31305" yWindow="165" windowWidth="24750" windowHeight="15405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -369,11 +369,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,6 +679,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="255.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1839,77 +1865,77 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="2">
         <v>0.1051085887991936</v>
       </c>
-      <c r="G17">
-        <v>31.89999961853027</v>
-      </c>
-      <c r="H17">
+      <c r="G17" s="2">
+        <v>30.10000038146973</v>
+      </c>
+      <c r="H17" s="2">
         <v>4346078.2796199042</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J17">
-        <v>3.3529639425985311</v>
-      </c>
-      <c r="K17">
+      <c r="J17" s="2">
+        <v>3.1637685629514722</v>
+      </c>
+      <c r="K17" s="2">
         <v>0.85161522344848883</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="2">
         <v>7.226800500286398</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="2">
         <v>-7.7720757767721924E-3</v>
       </c>
-      <c r="N17">
+      <c r="N17" s="2">
         <v>-0.77720757767721915</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="2">
         <v>0.86020631566819938</v>
       </c>
-      <c r="P17">
+      <c r="P17" s="2">
         <v>7.7939026203439399E-2</v>
       </c>
-      <c r="Q17">
+      <c r="Q17" s="2">
         <v>2.0764013992004702</v>
       </c>
-      <c r="R17">
+      <c r="R17" s="2">
         <v>15874.37</v>
       </c>
-      <c r="S17">
+      <c r="S17" s="2">
         <v>19092.2</v>
       </c>
-      <c r="T17">
+      <c r="T17" s="2">
         <v>1.2027059971513829</v>
       </c>
-      <c r="U17">
+      <c r="U17" s="2">
         <v>678.84</v>
       </c>
-      <c r="V17">
+      <c r="V17" s="2">
         <v>4.4340341999999998E-2</v>
       </c>
-      <c r="W17">
+      <c r="W17" s="2">
         <v>1.403</v>
       </c>
-      <c r="X17" t="s">
+      <c r="X17" s="2" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1933,7 +1959,7 @@
         <v>0.1051085887991936</v>
       </c>
       <c r="G18">
-        <v>1.1000000238418579</v>
+        <v>1.049999952316284</v>
       </c>
       <c r="H18">
         <v>12293773.82828456</v>
@@ -1942,7 +1968,7 @@
         <v>58</v>
       </c>
       <c r="J18">
-        <v>0.11561945018509701</v>
+        <v>0.11036401322718518</v>
       </c>
       <c r="K18">
         <v>6.6407358920662948E-2</v>

</xml_diff>